<commit_message>
QLDA: fix(du-an): bổ sung filter dashboard cho API theo dõi phòng phân công
Thêm thoiGianKhoiCong/thoiGianHoanThanh vào SearchDto và BuildQuery (pattern DuAnGetDanhSachQuery) để counter 4 panel và danh sách khớp filter dashboard; kèm issue docs
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/ExportTemplates/DanhSachTongHopVanBanQuyetDinh.xlsx
+++ b/QLDA.WebApi/ExportTemplates/DanhSachTongHopVanBanQuyetDinh.xlsx
@@ -16,10 +16,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
-    <t>Trung tâm chuyển đổi số thành phố Hồ Chí Minh</t>
-  </si>
-  <si>
-    <t>VĂN BẢN - QUYẾT ĐỊNH</t>
+    <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
+TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
+  </si>
+  <si>
+    <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
+Độc lập - Tự do - Hạnh phúc
+---------------</t>
+  </si>
+  <si>
+    <t>TỔNG HỢP VĂN BẢN QUYẾT ĐỊNH</t>
   </si>
   <si>
     <t>STT</t>
@@ -40,30 +46,31 @@
     <t>Trích yếu</t>
   </si>
   <si>
-    <t>$stt</t>
-  </si>
-  <si>
-    <t>$tenDuAn</t>
-  </si>
-  <si>
-    <t>$so</t>
-  </si>
-  <si>
-    <t>$ngay</t>
-  </si>
-  <si>
-    <t>$loai</t>
-  </si>
-  <si>
-    <t>$trichYeu</t>
+    <t>$Stt</t>
+  </si>
+  <si>
+    <t>$TenDuAn</t>
+  </si>
+  <si>
+    <t>$So</t>
+  </si>
+  <si>
+    <t>$Ngay</t>
+  </si>
+  <si>
+    <t>$Loai</t>
+  </si>
+  <si>
+    <t>$TrichYeu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="0" formatCode=""/>
+    <numFmt numFmtId="164" formatCode="dd/MM/yyyy"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -91,19 +98,24 @@
     <font>
       <b/>
       <vertAlign val="baseline"/>
-      <sz val="20"/>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="0" diagonalDown="0">
@@ -141,7 +153,7 @@
       </diagonal>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <protection locked="1" hidden="0"/>
     </xf>
@@ -154,10 +166,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection locked="1" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection locked="1" hidden="0"/>
     </xf>
   </cellStyleXfs>
@@ -174,32 +189,32 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
     </xf>
   </cellXfs>
@@ -497,88 +512,93 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="16384" width="9.140625" style="1" customWidth="1"/>
     <col min="1" max="1" width="6.710625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.710625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.710625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.710625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="22.710625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="35.710625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.710625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.710625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="32.710625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="39.710625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="49.710625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" customHeight="1">
+    <row r="1" spans="1:6" ht="36" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="B2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="32" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="5"/>
+    <row r="3" spans="1:6" ht="28" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="B4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="6" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>13</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="E1:F2"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A4:F4"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>